<commit_message>
P02c: truth currency, foreign-claim scale, scenario magnitudes, record numbering
Truth: every money column declares its currency (truth/money_columns.csv),
ultimates gain fx_cutoff_rate and earned_premium_try_at_cutoff_rate,
frequency_severity severities are named _try.
Fix: a foreign claim's cost was divided by the starting rate twice, so USD and
EUR claims were 2.95 and 3.25 times too small against their premium.
Scenarios: high_inflation and large_loss parameters retuned; new optional
line option large_events (rate per exposure year). Baseline output unchanged.
Records: 0007 specification format renumbered 0020; new record 0021.
</commit_message>
<xml_diff>
--- a/examples/baseline/claim_valuations.xlsx
+++ b/examples/baseline/claim_valuations.xlsx
@@ -11072,32 +11072,32 @@
         <v>0</v>
       </c>
       <c r="D262">
+        <v>0.09</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G262">
+        <v>0</v>
+      </c>
+      <c r="H262">
+        <v>0</v>
+      </c>
+      <c r="I262">
+        <v>0</v>
+      </c>
+      <c r="J262">
+        <v>0</v>
+      </c>
+      <c r="K262">
         <v>0.03</v>
-      </c>
-      <c r="E262" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="F262" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G262">
-        <v>0</v>
-      </c>
-      <c r="H262">
-        <v>0</v>
-      </c>
-      <c r="I262">
-        <v>0</v>
-      </c>
-      <c r="J262">
-        <v>0</v>
-      </c>
-      <c r="K262">
-        <v>0.01</v>
       </c>
     </row>
     <row r="263">
@@ -11930,10 +11930,10 @@
         <v>45107</v>
       </c>
       <c r="C283">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="D283">
-        <v>0.03</v>
+        <v>0.08</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -11958,7 +11958,7 @@
         <v>0</v>
       </c>
       <c r="K283">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="284">
@@ -12873,32 +12873,32 @@
         <v>45138</v>
       </c>
       <c r="C306">
+        <v>0.13</v>
+      </c>
+      <c r="D306">
+        <v>0</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>CLOSED</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="G306">
+        <v>0</v>
+      </c>
+      <c r="H306">
+        <v>0</v>
+      </c>
+      <c r="I306">
+        <v>0</v>
+      </c>
+      <c r="J306">
         <v>0.04</v>
-      </c>
-      <c r="D306">
-        <v>0</v>
-      </c>
-      <c r="E306" t="inlineStr">
-        <is>
-          <t>CLOSED</t>
-        </is>
-      </c>
-      <c r="F306" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="G306">
-        <v>0</v>
-      </c>
-      <c r="H306">
-        <v>0</v>
-      </c>
-      <c r="I306">
-        <v>0</v>
-      </c>
-      <c r="J306">
-        <v>0.01</v>
       </c>
       <c r="K306">
         <v>0</v>

</xml_diff>